<commit_message>
Rebuild from live sheet: 783 words, 502 learned (10 newly learned)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015idYdjgDV2QSzaddNufWAt
</commit_message>
<xml_diff>
--- a/japanese_n5_vocabulary_updated.xlsx
+++ b/japanese_n5_vocabulary_updated.xlsx
@@ -987,15 +987,15 @@
       </c>
       <c r="I2" s="57" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J2" s="57" t="n">
-        <v>82.5</v>
+        <v>99.5</v>
       </c>
       <c r="K2" s="57" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -1093,15 +1093,15 @@
       <c r="H4" s="57" t="n"/>
       <c r="I4" s="57" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J4" s="57" t="n">
-        <v>82.5</v>
+        <v>99.5</v>
       </c>
       <c r="K4" s="57" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -1144,15 +1144,15 @@
       <c r="H5" s="57" t="n"/>
       <c r="I5" s="57" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J5" s="57" t="n">
-        <v>82.5</v>
+        <v>99.5</v>
       </c>
       <c r="K5" s="57" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -1254,15 +1254,15 @@
       </c>
       <c r="I7" s="57" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J7" s="57" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K7" s="57" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -1309,15 +1309,15 @@
       </c>
       <c r="I8" s="57" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J8" s="57" t="n">
-        <v>82.5</v>
+        <v>99.5</v>
       </c>
       <c r="K8" s="57" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -1364,15 +1364,15 @@
       </c>
       <c r="I9" s="57" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="J9" s="57" t="n">
-        <v>82.5</v>
+        <v>99.5</v>
       </c>
       <c r="K9" s="57" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -1733,15 +1733,15 @@
       </c>
       <c r="I16" s="57" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="J16" s="57" t="n">
-        <v>72.40000000000001</v>
+        <v>86.5</v>
       </c>
       <c r="K16" s="57" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -1996,15 +1996,15 @@
       </c>
       <c r="I21" s="57" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J21" s="57" t="n">
-        <v>81.8</v>
+        <v>100</v>
       </c>
       <c r="K21" s="57" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -2149,15 +2149,15 @@
       <c r="H24" s="57" t="n"/>
       <c r="I24" s="57" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="J24" s="57" t="n">
-        <v>74.7</v>
+        <v>88</v>
       </c>
       <c r="K24" s="57" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -2204,15 +2204,15 @@
       </c>
       <c r="I25" s="57" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="J25" s="57" t="n">
-        <v>68.2</v>
+        <v>78.7</v>
       </c>
       <c r="K25" s="57" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -2314,15 +2314,15 @@
       </c>
       <c r="I27" s="57" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J27" s="57" t="n">
-        <v>82.5</v>
+        <v>99.5</v>
       </c>
       <c r="K27" s="57" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -2369,15 +2369,15 @@
       </c>
       <c r="I28" s="57" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="J28" s="57" t="n">
-        <v>74.7</v>
+        <v>88</v>
       </c>
       <c r="K28" s="57" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -2424,15 +2424,15 @@
       </c>
       <c r="I29" s="57" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="J29" s="57" t="n">
-        <v>74.7</v>
+        <v>88</v>
       </c>
       <c r="K29" s="57" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -2479,15 +2479,15 @@
       </c>
       <c r="I30" s="57" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="J30" s="57" t="n">
-        <v>82.5</v>
+        <v>99.5</v>
       </c>
       <c r="K30" s="57" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -2534,15 +2534,15 @@
       </c>
       <c r="I31" s="57" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="J31" s="57" t="n">
-        <v>66.8</v>
+        <v>77.7</v>
       </c>
       <c r="K31" s="57" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -2636,15 +2636,15 @@
       <c r="H33" s="57" t="n"/>
       <c r="I33" s="57" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J33" s="57" t="n">
-        <v>82.5</v>
+        <v>99.5</v>
       </c>
       <c r="K33" s="57" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -2687,15 +2687,15 @@
       <c r="H34" s="57" t="n"/>
       <c r="I34" s="57" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J34" s="57" t="n">
-        <v>82.5</v>
+        <v>99.5</v>
       </c>
       <c r="K34" s="57" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -2738,15 +2738,15 @@
       <c r="H35" s="57" t="n"/>
       <c r="I35" s="57" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="J35" s="57" t="n">
-        <v>82.5</v>
+        <v>99.5</v>
       </c>
       <c r="K35" s="57" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -3005,15 +3005,15 @@
       <c r="H40" s="57" t="n"/>
       <c r="I40" s="57" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J40" s="57" t="n">
-        <v>82.5</v>
+        <v>99.5</v>
       </c>
       <c r="K40" s="57" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -3056,15 +3056,15 @@
       <c r="H41" s="57" t="n"/>
       <c r="I41" s="57" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J41" s="57" t="n">
-        <v>82.5</v>
+        <v>99.5</v>
       </c>
       <c r="K41" s="57" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -3158,15 +3158,15 @@
       <c r="H43" s="57" t="n"/>
       <c r="I43" s="57" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J43" s="57" t="n">
-        <v>82.5</v>
+        <v>99.5</v>
       </c>
       <c r="K43" s="57" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -3209,15 +3209,15 @@
       <c r="H44" s="57" t="n"/>
       <c r="I44" s="57" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J44" s="57" t="n">
-        <v>80.40000000000001</v>
+        <v>98.40000000000001</v>
       </c>
       <c r="K44" s="57" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -3311,15 +3311,15 @@
       <c r="H46" s="57" t="n"/>
       <c r="I46" s="57" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J46" s="57" t="n">
-        <v>74.7</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="K46" s="57" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -3362,15 +3362,15 @@
       <c r="H47" s="57" t="n"/>
       <c r="I47" s="57" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="J47" s="57" t="n">
-        <v>82.5</v>
+        <v>99.5</v>
       </c>
       <c r="K47" s="57" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -3417,15 +3417,15 @@
       </c>
       <c r="I48" s="57" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="J48" s="57" t="n">
-        <v>71.09999999999999</v>
+        <v>80.7</v>
       </c>
       <c r="K48" s="57" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -3472,15 +3472,15 @@
       </c>
       <c r="I49" s="57" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="J49" s="57" t="n">
-        <v>74.7</v>
+        <v>88</v>
       </c>
       <c r="K49" s="57" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -3527,7 +3527,7 @@
       </c>
       <c r="I50" s="57" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J50" s="57" t="n">
@@ -3743,15 +3743,15 @@
       <c r="H54" s="57" t="n"/>
       <c r="I54" s="57" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="J54" s="57" t="n">
-        <v>68.2</v>
+        <v>78.7</v>
       </c>
       <c r="K54" s="57" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -3853,7 +3853,7 @@
       </c>
       <c r="I56" s="57" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J56" s="57" t="n">
@@ -3963,15 +3963,15 @@
       </c>
       <c r="I58" s="57" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="J58" s="57" t="n">
-        <v>74.7</v>
+        <v>88</v>
       </c>
       <c r="K58" s="57" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -4124,15 +4124,15 @@
       <c r="H61" s="57" t="n"/>
       <c r="I61" s="57" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J61" s="57" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K61" s="57" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -4230,15 +4230,15 @@
       <c r="H63" s="59" t="n"/>
       <c r="I63" s="59" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="J63" s="59" t="n">
-        <v>82.5</v>
+        <v>92.5</v>
       </c>
       <c r="K63" s="59" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -4336,15 +4336,15 @@
       <c r="H65" s="59" t="n"/>
       <c r="I65" s="59" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J65" s="59" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K65" s="59" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -4933,15 +4933,15 @@
       <c r="H76" s="60" t="n"/>
       <c r="I76" s="60" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J76" s="60" t="n">
-        <v>93.09999999999999</v>
+        <v>100</v>
       </c>
       <c r="K76" s="60" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -5416,15 +5416,15 @@
       </c>
       <c r="I85" s="61" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="J85" s="61" t="n">
-        <v>82.5</v>
+        <v>93.40000000000001</v>
       </c>
       <c r="K85" s="61" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -5636,15 +5636,15 @@
       </c>
       <c r="I89" s="61" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="J89" s="61" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K89" s="61" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -5746,15 +5746,15 @@
       </c>
       <c r="I91" s="61" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J91" s="61" t="n">
-        <v>62.3</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="K91" s="61" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -6021,15 +6021,15 @@
       </c>
       <c r="I96" s="62" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="J96" s="62" t="n">
-        <v>82.5</v>
+        <v>93.40000000000001</v>
       </c>
       <c r="K96" s="62" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -6296,7 +6296,7 @@
       </c>
       <c r="I101" s="63" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J101" s="63" t="n">
@@ -6406,15 +6406,15 @@
       </c>
       <c r="I103" s="63" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="J103" s="63" t="n">
-        <v>82.5</v>
+        <v>93.40000000000001</v>
       </c>
       <c r="K103" s="63" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -6681,7 +6681,7 @@
       </c>
       <c r="I108" s="63" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J108" s="63" t="n">
@@ -7121,15 +7121,15 @@
       </c>
       <c r="I116" s="64" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="J116" s="64" t="n">
-        <v>89.3</v>
+        <v>99.5</v>
       </c>
       <c r="K116" s="64" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -7176,15 +7176,15 @@
       </c>
       <c r="I117" s="64" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="J117" s="64" t="n">
-        <v>93.2</v>
+        <v>100</v>
       </c>
       <c r="K117" s="64" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -7231,15 +7231,15 @@
       </c>
       <c r="I118" s="64" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J118" s="64" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K118" s="64" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -7396,15 +7396,15 @@
       </c>
       <c r="I121" s="64" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="J121" s="64" t="n">
-        <v>94.90000000000001</v>
+        <v>98.09999999999999</v>
       </c>
       <c r="K121" s="64" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -7451,15 +7451,15 @@
       </c>
       <c r="I122" s="64" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J122" s="64" t="n">
-        <v>96.7</v>
+        <v>100</v>
       </c>
       <c r="K122" s="64" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -7726,15 +7726,15 @@
       </c>
       <c r="I127" s="65" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="J127" s="65" t="n">
-        <v>85</v>
+        <v>94.90000000000001</v>
       </c>
       <c r="K127" s="65" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -7891,15 +7891,15 @@
       </c>
       <c r="I130" s="65" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J130" s="65" t="n">
-        <v>93.09999999999999</v>
+        <v>99.5</v>
       </c>
       <c r="K130" s="65" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -8331,15 +8331,15 @@
       </c>
       <c r="I138" s="65" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="J138" s="65" t="n">
-        <v>81.59999999999999</v>
+        <v>88.7</v>
       </c>
       <c r="K138" s="65" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -8771,15 +8771,15 @@
       </c>
       <c r="I146" s="65" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="J146" s="65" t="n">
-        <v>70.09999999999999</v>
+        <v>85.09999999999999</v>
       </c>
       <c r="K146" s="65" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -9431,15 +9431,15 @@
       </c>
       <c r="I158" s="66" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J158" s="66" t="n">
-        <v>82.5</v>
+        <v>98.09999999999999</v>
       </c>
       <c r="K158" s="66" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -9596,15 +9596,15 @@
       </c>
       <c r="I161" s="66" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J161" s="66" t="n">
-        <v>67.3</v>
+        <v>80.90000000000001</v>
       </c>
       <c r="K161" s="66" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -9871,15 +9871,15 @@
       </c>
       <c r="I166" s="66" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J166" s="66" t="n">
-        <v>79.2</v>
+        <v>97.8</v>
       </c>
       <c r="K166" s="66" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -9926,15 +9926,15 @@
       </c>
       <c r="I167" s="66" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="J167" s="66" t="n">
-        <v>68.7</v>
+        <v>78.5</v>
       </c>
       <c r="K167" s="66" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -10091,15 +10091,15 @@
       </c>
       <c r="I170" s="66" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="J170" s="66" t="n">
-        <v>72.8</v>
+        <v>79.2</v>
       </c>
       <c r="K170" s="66" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -10421,15 +10421,15 @@
       </c>
       <c r="I176" s="66" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J176" s="66" t="n">
-        <v>87.2</v>
+        <v>99.5</v>
       </c>
       <c r="K176" s="66" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -10476,15 +10476,15 @@
       </c>
       <c r="I177" s="66" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J177" s="66" t="n">
-        <v>93.3</v>
+        <v>99.59999999999999</v>
       </c>
       <c r="K177" s="66" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -10751,15 +10751,15 @@
       </c>
       <c r="I182" s="66" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J182" s="66" t="n">
-        <v>64.3</v>
+        <v>73.8</v>
       </c>
       <c r="K182" s="66" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -10861,15 +10861,15 @@
       </c>
       <c r="I184" s="66" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="J184" s="66" t="n">
-        <v>87.2</v>
+        <v>100</v>
       </c>
       <c r="K184" s="66" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -11026,15 +11026,15 @@
       </c>
       <c r="I187" s="66" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="J187" s="66" t="n">
-        <v>82.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="K187" s="66" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -11191,15 +11191,15 @@
       </c>
       <c r="I190" s="66" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="J190" s="66" t="n">
-        <v>88.2</v>
+        <v>98.7</v>
       </c>
       <c r="K190" s="66" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -11411,15 +11411,15 @@
       </c>
       <c r="I194" s="66" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="J194" s="66" t="n">
-        <v>91.3</v>
+        <v>100</v>
       </c>
       <c r="K194" s="66" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -11466,15 +11466,15 @@
       </c>
       <c r="I195" s="66" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="J195" s="66" t="n">
-        <v>89.3</v>
+        <v>100</v>
       </c>
       <c r="K195" s="66" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -11521,15 +11521,15 @@
       </c>
       <c r="I196" s="66" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="J196" s="66" t="n">
-        <v>89.3</v>
+        <v>96.5</v>
       </c>
       <c r="K196" s="66" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -11631,15 +11631,15 @@
       </c>
       <c r="I198" s="66" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J198" s="66" t="n">
-        <v>91.3</v>
+        <v>98.09999999999999</v>
       </c>
       <c r="K198" s="66" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -11851,15 +11851,15 @@
       </c>
       <c r="I202" s="66" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="J202" s="66" t="n">
-        <v>81.59999999999999</v>
+        <v>86.5</v>
       </c>
       <c r="K202" s="66" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -11906,15 +11906,15 @@
       </c>
       <c r="I203" s="66" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="J203" s="66" t="n">
-        <v>82.5</v>
+        <v>91.3</v>
       </c>
       <c r="K203" s="66" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -12181,15 +12181,15 @@
       </c>
       <c r="I208" s="66" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="J208" s="66" t="n">
-        <v>89.3</v>
+        <v>94.90000000000001</v>
       </c>
       <c r="K208" s="66" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -12456,15 +12456,15 @@
       </c>
       <c r="I213" s="67" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="J213" s="67" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K213" s="67" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -12566,15 +12566,15 @@
       </c>
       <c r="I215" s="67" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="J215" s="67" t="n">
-        <v>82.5</v>
+        <v>93.40000000000001</v>
       </c>
       <c r="K215" s="67" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -12621,15 +12621,15 @@
       </c>
       <c r="I216" s="67" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J216" s="67" t="n">
-        <v>82.5</v>
+        <v>55</v>
       </c>
       <c r="K216" s="67" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -12676,15 +12676,15 @@
       </c>
       <c r="I217" s="67" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J217" s="67" t="n">
-        <v>82.5</v>
+        <v>94.2</v>
       </c>
       <c r="K217" s="67" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -12731,15 +12731,15 @@
       </c>
       <c r="I218" s="67" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J218" s="67" t="n">
-        <v>82.5</v>
+        <v>94.2</v>
       </c>
       <c r="K218" s="67" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -12841,15 +12841,15 @@
       </c>
       <c r="I220" s="67" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J220" s="67" t="n">
-        <v>65.3</v>
+        <v>74.5</v>
       </c>
       <c r="K220" s="67" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -12896,7 +12896,7 @@
       </c>
       <c r="I221" s="67" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J221" s="67" t="n">
@@ -13006,15 +13006,15 @@
       </c>
       <c r="I223" s="67" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="J223" s="67" t="n">
-        <v>69.8</v>
+        <v>98.09999999999999</v>
       </c>
       <c r="K223" s="67" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -13061,15 +13061,15 @@
       </c>
       <c r="I224" s="67" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J224" s="67" t="n">
-        <v>64</v>
+        <v>96</v>
       </c>
       <c r="K224" s="67" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -13116,15 +13116,15 @@
       </c>
       <c r="I225" s="67" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="J225" s="67" t="n">
-        <v>66.2</v>
+        <v>86.8</v>
       </c>
       <c r="K225" s="67" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -13171,15 +13171,15 @@
       </c>
       <c r="I226" s="67" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="J226" s="67" t="n">
-        <v>69.8</v>
+        <v>87.2</v>
       </c>
       <c r="K226" s="67" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -13391,15 +13391,15 @@
       </c>
       <c r="I230" s="67" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="J230" s="67" t="n">
-        <v>60.6</v>
+        <v>80.7</v>
       </c>
       <c r="K230" s="67" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -13501,7 +13501,7 @@
       </c>
       <c r="I232" s="67" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J232" s="67" t="n">
@@ -13611,15 +13611,15 @@
       </c>
       <c r="I234" s="67" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="J234" s="67" t="n">
-        <v>66.2</v>
+        <v>86.8</v>
       </c>
       <c r="K234" s="67" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -13666,15 +13666,15 @@
       </c>
       <c r="I235" s="67" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="J235" s="67" t="n">
-        <v>77.40000000000001</v>
+        <v>100</v>
       </c>
       <c r="K235" s="67" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -13721,15 +13721,15 @@
       </c>
       <c r="I236" s="67" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J236" s="67" t="n">
-        <v>66.2</v>
+        <v>92.2</v>
       </c>
       <c r="K236" s="67" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -14161,15 +14161,15 @@
       </c>
       <c r="I244" s="67" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="J244" s="67" t="n">
-        <v>66.2</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="K244" s="67" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -14381,15 +14381,15 @@
       </c>
       <c r="I248" s="67" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="J248" s="67" t="n">
-        <v>69</v>
+        <v>90.90000000000001</v>
       </c>
       <c r="K248" s="67" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -14436,15 +14436,15 @@
       </c>
       <c r="I249" s="67" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J249" s="67" t="n">
-        <v>66.2</v>
+        <v>92.2</v>
       </c>
       <c r="K249" s="67" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -15096,15 +15096,15 @@
       </c>
       <c r="I261" s="67" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="J261" s="67" t="n">
-        <v>41.4</v>
+        <v>61.1</v>
       </c>
       <c r="K261" s="67" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -15206,15 +15206,15 @@
       </c>
       <c r="I263" s="67" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="J263" s="67" t="n">
-        <v>55.4</v>
+        <v>82</v>
       </c>
       <c r="K263" s="67" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -15261,15 +15261,15 @@
       </c>
       <c r="I264" s="67" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J264" s="67" t="n">
-        <v>66.8</v>
+        <v>83.2</v>
       </c>
       <c r="K264" s="67" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -15536,15 +15536,15 @@
       </c>
       <c r="I269" s="67" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J269" s="67" t="n">
-        <v>40.4</v>
+        <v>60.6</v>
       </c>
       <c r="K269" s="67" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -15811,15 +15811,15 @@
       </c>
       <c r="I274" s="67" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="J274" s="67" t="n">
-        <v>67.09999999999999</v>
+        <v>92.5</v>
       </c>
       <c r="K274" s="67" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -15921,15 +15921,15 @@
       </c>
       <c r="I276" s="67" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="J276" s="67" t="n">
-        <v>62</v>
+        <v>81.5</v>
       </c>
       <c r="K276" s="67" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -16196,7 +16196,7 @@
       </c>
       <c r="I281" s="67" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J281" s="67" t="n">
@@ -16361,15 +16361,15 @@
       </c>
       <c r="I284" s="67" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J284" s="67" t="n">
-        <v>62</v>
+        <v>84.8</v>
       </c>
       <c r="K284" s="67" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -16471,15 +16471,15 @@
       </c>
       <c r="I286" s="67" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="J286" s="67" t="n">
-        <v>56.7</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="K286" s="67" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -16581,15 +16581,15 @@
       </c>
       <c r="I288" s="67" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="J288" s="67" t="n">
-        <v>40.4</v>
+        <v>60.6</v>
       </c>
       <c r="K288" s="67" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -16691,15 +16691,15 @@
       </c>
       <c r="I290" s="67" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="J290" s="67" t="n">
-        <v>62</v>
+        <v>74.5</v>
       </c>
       <c r="K290" s="67" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -17571,15 +17571,15 @@
       </c>
       <c r="I306" s="67" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J306" s="67" t="n">
-        <v>66.2</v>
+        <v>56.8</v>
       </c>
       <c r="K306" s="67" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -17956,15 +17956,15 @@
       </c>
       <c r="I313" s="67" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J313" s="67" t="n">
-        <v>53.1</v>
+        <v>72.8</v>
       </c>
       <c r="K313" s="67" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -18231,15 +18231,15 @@
       </c>
       <c r="I318" s="67" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="J318" s="67" t="n">
-        <v>71.90000000000001</v>
+        <v>75.09999999999999</v>
       </c>
       <c r="K318" s="67" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -19166,15 +19166,15 @@
       </c>
       <c r="I335" s="67" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="J335" s="67" t="n">
-        <v>54.5</v>
+        <v>60.2</v>
       </c>
       <c r="K335" s="67" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -19716,15 +19716,15 @@
       </c>
       <c r="I345" s="68" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J345" s="68" t="n">
-        <v>67.3</v>
+        <v>80.90000000000001</v>
       </c>
       <c r="K345" s="68" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -19771,15 +19771,15 @@
       </c>
       <c r="I346" s="68" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J346" s="68" t="n">
-        <v>82.5</v>
+        <v>99.5</v>
       </c>
       <c r="K346" s="68" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -20046,15 +20046,15 @@
       </c>
       <c r="I351" s="68" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J351" s="68" t="n">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="K351" s="68" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -20321,15 +20321,15 @@
       </c>
       <c r="I356" s="68" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J356" s="68" t="n">
-        <v>82.5</v>
+        <v>91.3</v>
       </c>
       <c r="K356" s="68" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -20431,15 +20431,15 @@
       </c>
       <c r="I358" s="68" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J358" s="68" t="n">
-        <v>76.40000000000001</v>
+        <v>86.90000000000001</v>
       </c>
       <c r="K358" s="68" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -20486,15 +20486,15 @@
       </c>
       <c r="I359" s="68" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="J359" s="68" t="n">
-        <v>82.5</v>
+        <v>93.09999999999999</v>
       </c>
       <c r="K359" s="68" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -20651,15 +20651,15 @@
       </c>
       <c r="I362" s="69" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J362" s="69" t="n">
-        <v>47.6</v>
+        <v>57.6</v>
       </c>
       <c r="K362" s="69" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -20761,15 +20761,15 @@
       </c>
       <c r="I364" s="69" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J364" s="69" t="n">
-        <v>60.6</v>
+        <v>69.3</v>
       </c>
       <c r="K364" s="69" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -21256,15 +21256,15 @@
       </c>
       <c r="I373" s="69" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="J373" s="69" t="n">
-        <v>93.09999999999999</v>
+        <v>98.09999999999999</v>
       </c>
       <c r="K373" s="69" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -21311,15 +21311,15 @@
       </c>
       <c r="I374" s="69" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J374" s="69" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K374" s="69" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -21531,15 +21531,15 @@
       </c>
       <c r="I378" s="69" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J378" s="69" t="n">
-        <v>93.09999999999999</v>
+        <v>100</v>
       </c>
       <c r="K378" s="69" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -22136,15 +22136,15 @@
       </c>
       <c r="I389" s="69" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="J389" s="69" t="n">
-        <v>64.3</v>
+        <v>79.09999999999999</v>
       </c>
       <c r="K389" s="69" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -22411,15 +22411,15 @@
       </c>
       <c r="I394" s="69" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J394" s="69" t="n">
-        <v>64.3</v>
+        <v>73.8</v>
       </c>
       <c r="K394" s="69" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -22466,15 +22466,15 @@
       </c>
       <c r="I395" s="69" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="J395" s="69" t="n">
-        <v>85</v>
+        <v>96.5</v>
       </c>
       <c r="K395" s="69" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -22521,15 +22521,15 @@
       </c>
       <c r="I396" s="69" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="J396" s="69" t="n">
-        <v>94.90000000000001</v>
+        <v>99.5</v>
       </c>
       <c r="K396" s="69" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -22576,15 +22576,15 @@
       </c>
       <c r="I397" s="69" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J397" s="69" t="n">
-        <v>91.3</v>
+        <v>99.5</v>
       </c>
       <c r="K397" s="69" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -23016,15 +23016,15 @@
       </c>
       <c r="I405" s="69" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="J405" s="69" t="n">
-        <v>69.8</v>
+        <v>79.2</v>
       </c>
       <c r="K405" s="69" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -23291,15 +23291,15 @@
       </c>
       <c r="I410" s="69" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="J410" s="69" t="n">
-        <v>69.8</v>
+        <v>79.2</v>
       </c>
       <c r="K410" s="69" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -24226,15 +24226,15 @@
       </c>
       <c r="I427" s="70" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="J427" s="70" t="n">
-        <v>73.8</v>
+        <v>80</v>
       </c>
       <c r="K427" s="70" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -24281,15 +24281,15 @@
       </c>
       <c r="I428" s="70" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="J428" s="70" t="n">
-        <v>69.8</v>
+        <v>91.3</v>
       </c>
       <c r="K428" s="70" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -24446,15 +24446,15 @@
       </c>
       <c r="I431" s="70" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="J431" s="70" t="n">
-        <v>69.8</v>
+        <v>91.3</v>
       </c>
       <c r="K431" s="70" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -24831,15 +24831,15 @@
       </c>
       <c r="I438" s="70" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="J438" s="70" t="n">
-        <v>93.09999999999999</v>
+        <v>98.09999999999999</v>
       </c>
       <c r="K438" s="70" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -24996,15 +24996,15 @@
       </c>
       <c r="I441" s="70" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="J441" s="70" t="n">
-        <v>74.7</v>
+        <v>98.09999999999999</v>
       </c>
       <c r="K441" s="70" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -25106,15 +25106,15 @@
       </c>
       <c r="I443" s="70" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J443" s="70" t="n">
-        <v>90.59999999999999</v>
+        <v>99</v>
       </c>
       <c r="K443" s="70" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -25436,15 +25436,15 @@
       </c>
       <c r="I449" s="70" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="J449" s="70" t="n">
-        <v>59.8</v>
+        <v>80.40000000000001</v>
       </c>
       <c r="K449" s="70" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -25546,15 +25546,15 @@
       </c>
       <c r="I451" s="70" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="J451" s="70" t="n">
-        <v>77.90000000000001</v>
+        <v>88</v>
       </c>
       <c r="K451" s="70" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -25711,15 +25711,15 @@
       </c>
       <c r="I454" s="70" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="J454" s="70" t="n">
-        <v>60.9</v>
+        <v>77.09999999999999</v>
       </c>
       <c r="K454" s="70" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -25766,15 +25766,15 @@
       </c>
       <c r="I455" s="70" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J455" s="70" t="n">
-        <v>77.90000000000001</v>
+        <v>85.7</v>
       </c>
       <c r="K455" s="70" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -25821,15 +25821,15 @@
       </c>
       <c r="I456" s="70" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="J456" s="70" t="n">
-        <v>87.90000000000001</v>
+        <v>93.7</v>
       </c>
       <c r="K456" s="70" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -25876,15 +25876,15 @@
       </c>
       <c r="I457" s="70" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="J457" s="70" t="n">
-        <v>69.8</v>
+        <v>91.3</v>
       </c>
       <c r="K457" s="70" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -26151,15 +26151,15 @@
       </c>
       <c r="I462" s="70" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J462" s="70" t="n">
-        <v>96.7</v>
+        <v>100</v>
       </c>
       <c r="K462" s="70" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -26206,15 +26206,15 @@
       </c>
       <c r="I463" s="70" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J463" s="70" t="n">
-        <v>88.40000000000001</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="K463" s="70" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -26426,15 +26426,15 @@
       </c>
       <c r="I467" s="70" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="J467" s="70" t="n">
-        <v>82.5</v>
+        <v>96.5</v>
       </c>
       <c r="K467" s="70" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -26481,15 +26481,15 @@
       </c>
       <c r="I468" s="70" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J468" s="70" t="n">
-        <v>96.7</v>
+        <v>100</v>
       </c>
       <c r="K468" s="70" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -26536,15 +26536,15 @@
       </c>
       <c r="I469" s="70" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="J469" s="70" t="n">
-        <v>93.09999999999999</v>
+        <v>99.5</v>
       </c>
       <c r="K469" s="70" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -26756,15 +26756,15 @@
       </c>
       <c r="I473" s="71" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="J473" s="71" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K473" s="71" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -27031,15 +27031,15 @@
       </c>
       <c r="I478" s="71" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J478" s="71" t="n">
-        <v>82.5</v>
+        <v>94.2</v>
       </c>
       <c r="K478" s="71" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -38373,15 +38373,15 @@
       <c r="H710" s="70" t="n"/>
       <c r="I710" s="70" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J710" s="70" t="n">
-        <v>40.4</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="K710" s="70" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -38551,15 +38551,15 @@
       <c r="H714" s="70" t="n"/>
       <c r="I714" s="70" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="J714" s="70" t="n">
-        <v>40.4</v>
+        <v>67.09999999999999</v>
       </c>
       <c r="K714" s="70" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -38913,15 +38913,15 @@
       <c r="H722" s="70" t="n"/>
       <c r="I722" s="70" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="J722" s="70" t="n">
-        <v>56.9</v>
+        <v>59.6</v>
       </c>
       <c r="K722" s="70" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -38999,17 +38999,23 @@
       </c>
       <c r="G724" s="34" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="H724" s="70" t="n"/>
       <c r="I724" s="70" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="J724" s="70" t="n"/>
-      <c r="K724" s="70" t="n"/>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="J724" s="70" t="n">
+        <v>41.1</v>
+      </c>
+      <c r="K724" s="70" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
     </row>
     <row r="725">
       <c r="A725" s="70" t="inlineStr">
@@ -39044,17 +39050,23 @@
       </c>
       <c r="G725" s="34" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="H725" s="70" t="n"/>
       <c r="I725" s="70" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="J725" s="70" t="n"/>
-      <c r="K725" s="70" t="n"/>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="J725" s="70" t="n">
+        <v>41.1</v>
+      </c>
+      <c r="K725" s="70" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
     </row>
     <row r="726">
       <c r="A726" s="70" t="inlineStr">
@@ -39130,17 +39142,23 @@
       </c>
       <c r="G727" s="34" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="H727" s="70" t="n"/>
       <c r="I727" s="70" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
-        </is>
-      </c>
-      <c r="J727" s="70" t="n"/>
-      <c r="K727" s="70" t="n"/>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="J727" s="70" t="n">
+        <v>41.1</v>
+      </c>
+      <c r="K727" s="70" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
     </row>
     <row r="728">
       <c r="A728" s="70" t="inlineStr">
@@ -39443,15 +39461,15 @@
       </c>
       <c r="I734" s="70" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="J734" s="70" t="n">
-        <v>28.9</v>
+        <v>49.6</v>
       </c>
       <c r="K734" s="70" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -39615,7 +39633,7 @@
       </c>
       <c r="G738" s="34" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="H738" s="70" t="inlineStr">
@@ -39625,11 +39643,17 @@
       </c>
       <c r="I738" s="70" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="J738" s="70" t="n"/>
-      <c r="K738" s="70" t="n"/>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="J738" s="70" t="n">
+        <v>20.2</v>
+      </c>
+      <c r="K738" s="70" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
     </row>
     <row r="739">
       <c r="A739" s="70" t="inlineStr">
@@ -39664,7 +39688,7 @@
       </c>
       <c r="G739" s="34" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="H739" s="70" t="inlineStr">
@@ -39674,11 +39698,17 @@
       </c>
       <c r="I739" s="70" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="J739" s="70" t="n"/>
-      <c r="K739" s="70" t="n"/>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="J739" s="70" t="n">
+        <v>20.2</v>
+      </c>
+      <c r="K739" s="70" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
     </row>
     <row r="740">
       <c r="A740" s="70" t="inlineStr">
@@ -39944,15 +39974,15 @@
       </c>
       <c r="I745" s="70" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="J745" s="70" t="n">
-        <v>28.9</v>
+        <v>49.6</v>
       </c>
       <c r="K745" s="70" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -39999,15 +40029,15 @@
       </c>
       <c r="I746" s="70" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="J746" s="70" t="n">
-        <v>28.9</v>
+        <v>49.6</v>
       </c>
       <c r="K746" s="70" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -40099,15 +40129,15 @@
       </c>
       <c r="I748" s="70" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="J748" s="70" t="n">
-        <v>28.9</v>
+        <v>49.6</v>
       </c>
       <c r="K748" s="70" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -40154,15 +40184,15 @@
       </c>
       <c r="I749" s="70" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="J749" s="70" t="n">
-        <v>28.9</v>
+        <v>49.6</v>
       </c>
       <c r="K749" s="70" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -40420,17 +40450,23 @@
       </c>
       <c r="G755" s="34" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="H755" s="70" t="n"/>
       <c r="I755" s="70" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
-        </is>
-      </c>
-      <c r="J755" s="70" t="n"/>
-      <c r="K755" s="70" t="n"/>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="J755" s="70" t="n">
+        <v>41.1</v>
+      </c>
+      <c r="K755" s="70" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
     </row>
     <row r="756">
       <c r="A756" s="70" t="inlineStr">
@@ -40569,15 +40605,15 @@
       </c>
       <c r="I758" s="70" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="J758" s="70" t="n">
-        <v>20.2</v>
+        <v>45.7</v>
       </c>
       <c r="K758" s="70" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -40823,13 +40859,23 @@
       </c>
       <c r="G764" s="34" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="H764" s="70" t="n"/>
-      <c r="I764" s="70" t="n"/>
-      <c r="J764" s="70" t="n"/>
-      <c r="K764" s="70" t="n"/>
+      <c r="I764" s="70" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="J764" s="70" t="n">
+        <v>20.2</v>
+      </c>
+      <c r="K764" s="70" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
     </row>
     <row r="765">
       <c r="A765" s="70" t="inlineStr">
@@ -40870,15 +40916,15 @@
       <c r="H765" s="70" t="n"/>
       <c r="I765" s="70" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="J765" s="70" t="n">
-        <v>56.9</v>
+        <v>59.6</v>
       </c>
       <c r="K765" s="70" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -40921,15 +40967,15 @@
       <c r="H766" s="70" t="n"/>
       <c r="I766" s="70" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="J766" s="70" t="n">
-        <v>47.2</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="K766" s="70" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -41048,13 +41094,23 @@
       </c>
       <c r="G769" s="34" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="H769" s="70" t="n"/>
-      <c r="I769" s="70" t="n"/>
-      <c r="J769" s="70" t="n"/>
-      <c r="K769" s="70" t="n"/>
+      <c r="I769" s="70" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="J769" s="70" t="n">
+        <v>20.2</v>
+      </c>
+      <c r="K769" s="70" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
     </row>
     <row r="770">
       <c r="A770" s="70" t="inlineStr">
@@ -41099,15 +41155,15 @@
       </c>
       <c r="I770" s="70" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="J770" s="70" t="n">
-        <v>35.6</v>
+        <v>53.1</v>
       </c>
       <c r="K770" s="70" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -41154,15 +41210,15 @@
       </c>
       <c r="I771" s="70" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="J771" s="70" t="n">
-        <v>20.2</v>
+        <v>52.7</v>
       </c>
       <c r="K771" s="70" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -41209,15 +41265,15 @@
       </c>
       <c r="I772" s="70" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="J772" s="70" t="n">
-        <v>35.6</v>
+        <v>56.7</v>
       </c>
       <c r="K772" s="70" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -41264,15 +41320,15 @@
       </c>
       <c r="I773" s="70" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="J773" s="70" t="n">
-        <v>45.1</v>
+        <v>58.7</v>
       </c>
       <c r="K773" s="70" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -41309,13 +41365,23 @@
       </c>
       <c r="G774" s="34" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="H774" s="70" t="n"/>
-      <c r="I774" s="70" t="n"/>
-      <c r="J774" s="70" t="n"/>
-      <c r="K774" s="70" t="n"/>
+      <c r="I774" s="70" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="J774" s="70" t="n">
+        <v>41.1</v>
+      </c>
+      <c r="K774" s="70" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
     </row>
     <row r="775">
       <c r="A775" s="70" t="inlineStr">
@@ -41350,13 +41416,23 @@
       </c>
       <c r="G775" s="34" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="H775" s="70" t="n"/>
-      <c r="I775" s="70" t="n"/>
-      <c r="J775" s="70" t="n"/>
-      <c r="K775" s="70" t="n"/>
+      <c r="I775" s="70" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
+      <c r="J775" s="70" t="n">
+        <v>20.2</v>
+      </c>
+      <c r="K775" s="70" t="inlineStr">
+        <is>
+          <t>2026-10-22</t>
+        </is>
+      </c>
     </row>
     <row r="776">
       <c r="A776" s="70" t="inlineStr">
@@ -41775,7 +41851,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>492</v>
+        <v>502</v>
       </c>
     </row>
     <row r="5">
@@ -41785,7 +41861,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>291</v>
+        <v>281</v>
       </c>
     </row>
     <row r="6">
@@ -41796,7 +41872,7 @@
       </c>
       <c r="B6" s="16" t="inlineStr">
         <is>
-          <t>62.8%</t>
+          <t>64.1%</t>
         </is>
       </c>
     </row>
@@ -41983,7 +42059,7 @@
         <v>119</v>
       </c>
       <c r="C21" t="n">
-        <v>66</v>
+        <v>76</v>
       </c>
     </row>
     <row r="22">

</xml_diff>

<commit_message>
Rebuild from live sheet (3cf159b): 783 words, 517 learned, no word changes
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015idYdjgDV2QSzaddNufWAt
</commit_message>
<xml_diff>
--- a/japanese_n5_vocabulary_updated.xlsx
+++ b/japanese_n5_vocabulary_updated.xlsx
@@ -1627,15 +1627,15 @@
       <c r="H14" s="57" t="n"/>
       <c r="I14" s="57" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J14" s="57" t="n">
-        <v>72.09999999999999</v>
+        <v>45.7</v>
       </c>
       <c r="K14" s="57" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -2204,15 +2204,15 @@
       </c>
       <c r="I25" s="57" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J25" s="57" t="n">
-        <v>78.7</v>
+        <v>100</v>
       </c>
       <c r="K25" s="57" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -4018,15 +4018,15 @@
       </c>
       <c r="I59" s="57" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J59" s="57" t="n">
-        <v>81.59999999999999</v>
+        <v>100</v>
       </c>
       <c r="K59" s="57" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -4827,15 +4827,15 @@
       </c>
       <c r="I74" s="60" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J74" s="60" t="n">
-        <v>73.09999999999999</v>
+        <v>100</v>
       </c>
       <c r="K74" s="60" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -4988,15 +4988,15 @@
       </c>
       <c r="I77" s="60" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J77" s="60" t="n">
-        <v>55</v>
+        <v>31.6</v>
       </c>
       <c r="K77" s="60" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -5200,15 +5200,15 @@
       </c>
       <c r="I81" s="60" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J81" s="60" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K81" s="60" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -5361,15 +5361,15 @@
       </c>
       <c r="I84" s="61" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J84" s="61" t="n">
-        <v>89.3</v>
+        <v>100</v>
       </c>
       <c r="K84" s="61" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -5471,15 +5471,15 @@
       </c>
       <c r="I86" s="61" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J86" s="61" t="n">
-        <v>68.5</v>
+        <v>99.5</v>
       </c>
       <c r="K86" s="61" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -5691,15 +5691,15 @@
       </c>
       <c r="I90" s="61" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J90" s="61" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K90" s="61" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -5746,15 +5746,15 @@
       </c>
       <c r="I91" s="61" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J91" s="61" t="n">
-        <v>72.40000000000001</v>
+        <v>94.90000000000001</v>
       </c>
       <c r="K91" s="61" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -5856,15 +5856,15 @@
       </c>
       <c r="I93" s="62" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J93" s="62" t="n">
-        <v>76.40000000000001</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="K93" s="62" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -6791,15 +6791,15 @@
       </c>
       <c r="I110" s="64" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J110" s="64" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K110" s="64" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -6901,15 +6901,15 @@
       </c>
       <c r="I112" s="64" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J112" s="64" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K112" s="64" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -8056,15 +8056,15 @@
       </c>
       <c r="I133" s="65" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J133" s="65" t="n">
-        <v>76.59999999999999</v>
+        <v>49.7</v>
       </c>
       <c r="K133" s="65" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -8606,15 +8606,15 @@
       </c>
       <c r="I143" s="65" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J143" s="65" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K143" s="65" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -9156,15 +9156,15 @@
       </c>
       <c r="I153" s="66" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J153" s="66" t="n">
-        <v>87.2</v>
+        <v>100</v>
       </c>
       <c r="K153" s="66" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -9761,15 +9761,15 @@
       </c>
       <c r="I164" s="66" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J164" s="66" t="n">
-        <v>91.3</v>
+        <v>100</v>
       </c>
       <c r="K164" s="66" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -10311,15 +10311,15 @@
       </c>
       <c r="I174" s="66" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J174" s="66" t="n">
-        <v>91.3</v>
+        <v>100</v>
       </c>
       <c r="K174" s="66" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -10586,15 +10586,15 @@
       </c>
       <c r="I179" s="66" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J179" s="66" t="n">
-        <v>85.7</v>
+        <v>100</v>
       </c>
       <c r="K179" s="66" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -11246,15 +11246,15 @@
       </c>
       <c r="I191" s="66" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J191" s="66" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K191" s="66" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -11741,15 +11741,15 @@
       </c>
       <c r="I200" s="66" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J200" s="66" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K200" s="66" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -12346,15 +12346,15 @@
       </c>
       <c r="I211" s="66" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J211" s="66" t="n">
-        <v>89.3</v>
+        <v>100</v>
       </c>
       <c r="K211" s="66" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -12401,15 +12401,15 @@
       </c>
       <c r="I212" s="66" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J212" s="66" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K212" s="66" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -12621,15 +12621,15 @@
       </c>
       <c r="I216" s="67" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J216" s="67" t="n">
-        <v>31.6</v>
+        <v>46.6</v>
       </c>
       <c r="K216" s="67" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -13336,15 +13336,15 @@
       </c>
       <c r="I229" s="67" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J229" s="67" t="n">
-        <v>74</v>
+        <v>100</v>
       </c>
       <c r="K229" s="67" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -13446,15 +13446,15 @@
       </c>
       <c r="I231" s="67" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J231" s="67" t="n">
-        <v>75.8</v>
+        <v>100</v>
       </c>
       <c r="K231" s="67" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -14821,15 +14821,15 @@
       </c>
       <c r="I256" s="67" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J256" s="67" t="n">
-        <v>82.5</v>
+        <v>55</v>
       </c>
       <c r="K256" s="67" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -14876,15 +14876,15 @@
       </c>
       <c r="I257" s="67" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J257" s="67" t="n">
-        <v>76.2</v>
+        <v>100</v>
       </c>
       <c r="K257" s="67" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -15041,15 +15041,15 @@
       </c>
       <c r="I260" s="67" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J260" s="67" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K260" s="67" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -15426,15 +15426,15 @@
       </c>
       <c r="I267" s="67" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J267" s="67" t="n">
-        <v>85.7</v>
+        <v>100</v>
       </c>
       <c r="K267" s="67" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -16141,15 +16141,15 @@
       </c>
       <c r="I280" s="67" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J280" s="67" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K280" s="67" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -16251,15 +16251,15 @@
       </c>
       <c r="I282" s="67" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J282" s="67" t="n">
-        <v>85.7</v>
+        <v>100</v>
       </c>
       <c r="K282" s="67" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -16306,15 +16306,15 @@
       </c>
       <c r="I283" s="67" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J283" s="67" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K283" s="67" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -16416,15 +16416,15 @@
       </c>
       <c r="I285" s="67" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J285" s="67" t="n">
-        <v>76.2</v>
+        <v>100</v>
       </c>
       <c r="K285" s="67" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -16636,15 +16636,15 @@
       </c>
       <c r="I289" s="67" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J289" s="67" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K289" s="67" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -16746,15 +16746,15 @@
       </c>
       <c r="I291" s="67" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J291" s="67" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K291" s="67" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -16801,15 +16801,15 @@
       </c>
       <c r="I292" s="67" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J292" s="67" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K292" s="67" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -17076,15 +17076,15 @@
       </c>
       <c r="I297" s="67" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J297" s="67" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K297" s="67" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -17406,15 +17406,15 @@
       </c>
       <c r="I303" s="67" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J303" s="67" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K303" s="67" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -17461,15 +17461,15 @@
       </c>
       <c r="I304" s="67" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J304" s="67" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K304" s="67" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -17516,15 +17516,15 @@
       </c>
       <c r="I305" s="67" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J305" s="67" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K305" s="67" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -17846,15 +17846,15 @@
       </c>
       <c r="I311" s="67" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J311" s="67" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K311" s="67" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -17956,15 +17956,15 @@
       </c>
       <c r="I313" s="67" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J313" s="67" t="n">
-        <v>72.8</v>
+        <v>95.09999999999999</v>
       </c>
       <c r="K313" s="67" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -18286,15 +18286,15 @@
       </c>
       <c r="I319" s="67" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J319" s="67" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K319" s="67" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -18341,15 +18341,15 @@
       </c>
       <c r="I320" s="67" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J320" s="67" t="n">
-        <v>68.5</v>
+        <v>99.5</v>
       </c>
       <c r="K320" s="67" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -18396,15 +18396,15 @@
       </c>
       <c r="I321" s="67" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J321" s="67" t="n">
-        <v>87.2</v>
+        <v>100</v>
       </c>
       <c r="K321" s="67" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -18616,15 +18616,15 @@
       </c>
       <c r="I325" s="67" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J325" s="67" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K325" s="67" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -18726,15 +18726,15 @@
       </c>
       <c r="I327" s="67" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J327" s="67" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K327" s="67" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -18781,15 +18781,15 @@
       </c>
       <c r="I328" s="67" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J328" s="67" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K328" s="67" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -18836,15 +18836,15 @@
       </c>
       <c r="I329" s="67" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J329" s="67" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K329" s="67" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -18891,15 +18891,15 @@
       </c>
       <c r="I330" s="67" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J330" s="67" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K330" s="67" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -19001,15 +19001,15 @@
       </c>
       <c r="I332" s="67" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J332" s="67" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K332" s="67" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -19111,15 +19111,15 @@
       </c>
       <c r="I334" s="67" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J334" s="67" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K334" s="67" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -19221,15 +19221,15 @@
       </c>
       <c r="I336" s="67" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J336" s="67" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K336" s="67" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -19276,15 +19276,15 @@
       </c>
       <c r="I337" s="67" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J337" s="67" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K337" s="67" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -20706,15 +20706,15 @@
       </c>
       <c r="I363" s="69" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J363" s="69" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K363" s="69" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -20761,15 +20761,15 @@
       </c>
       <c r="I364" s="69" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J364" s="69" t="n">
-        <v>69.3</v>
+        <v>43.3</v>
       </c>
       <c r="K364" s="69" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -20816,15 +20816,15 @@
       </c>
       <c r="I365" s="69" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J365" s="69" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K365" s="69" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -20871,15 +20871,15 @@
       </c>
       <c r="I366" s="69" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J366" s="69" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K366" s="69" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -20981,15 +20981,15 @@
       </c>
       <c r="I368" s="69" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J368" s="69" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K368" s="69" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -21036,15 +21036,15 @@
       </c>
       <c r="I369" s="69" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J369" s="69" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K369" s="69" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -21091,15 +21091,15 @@
       </c>
       <c r="I370" s="69" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J370" s="69" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K370" s="69" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -21146,15 +21146,15 @@
       </c>
       <c r="I371" s="69" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J371" s="69" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K371" s="69" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -21201,15 +21201,15 @@
       </c>
       <c r="I372" s="69" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J372" s="69" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K372" s="69" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -21366,15 +21366,15 @@
       </c>
       <c r="I375" s="69" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J375" s="69" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K375" s="69" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -21421,15 +21421,15 @@
       </c>
       <c r="I376" s="69" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J376" s="69" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K376" s="69" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -21476,15 +21476,15 @@
       </c>
       <c r="I377" s="69" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J377" s="69" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K377" s="69" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -21586,15 +21586,15 @@
       </c>
       <c r="I379" s="69" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J379" s="69" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K379" s="69" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -21641,15 +21641,15 @@
       </c>
       <c r="I380" s="69" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J380" s="69" t="n">
-        <v>77.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="K380" s="69" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -21696,15 +21696,15 @@
       </c>
       <c r="I381" s="69" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J381" s="69" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K381" s="69" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -21751,15 +21751,15 @@
       </c>
       <c r="I382" s="69" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J382" s="69" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K382" s="69" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -21861,15 +21861,15 @@
       </c>
       <c r="I384" s="69" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J384" s="69" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K384" s="69" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -21916,15 +21916,15 @@
       </c>
       <c r="I385" s="69" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J385" s="69" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K385" s="69" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -22081,15 +22081,15 @@
       </c>
       <c r="I388" s="69" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J388" s="69" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K388" s="69" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -22191,15 +22191,15 @@
       </c>
       <c r="I390" s="69" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J390" s="69" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K390" s="69" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -22301,15 +22301,15 @@
       </c>
       <c r="I392" s="69" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J392" s="69" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K392" s="69" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -22741,15 +22741,15 @@
       </c>
       <c r="I400" s="69" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J400" s="69" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K400" s="69" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -22796,15 +22796,15 @@
       </c>
       <c r="I401" s="69" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J401" s="69" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K401" s="69" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -22851,15 +22851,15 @@
       </c>
       <c r="I402" s="69" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J402" s="69" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K402" s="69" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -23071,15 +23071,15 @@
       </c>
       <c r="I406" s="69" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J406" s="69" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K406" s="69" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -23126,15 +23126,15 @@
       </c>
       <c r="I407" s="69" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J407" s="69" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K407" s="69" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -23181,15 +23181,15 @@
       </c>
       <c r="I408" s="69" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J408" s="69" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K408" s="69" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -23401,15 +23401,15 @@
       </c>
       <c r="I412" s="69" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J412" s="69" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K412" s="69" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -23456,15 +23456,15 @@
       </c>
       <c r="I413" s="69" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J413" s="69" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K413" s="69" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -23566,15 +23566,15 @@
       </c>
       <c r="I415" s="69" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J415" s="69" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K415" s="69" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -23621,15 +23621,15 @@
       </c>
       <c r="I416" s="69" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J416" s="69" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K416" s="69" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -23676,15 +23676,15 @@
       </c>
       <c r="I417" s="69" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J417" s="69" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K417" s="69" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -23731,15 +23731,15 @@
       </c>
       <c r="I418" s="69" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J418" s="69" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K418" s="69" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -23896,15 +23896,15 @@
       </c>
       <c r="I421" s="70" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J421" s="70" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K421" s="70" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -23951,15 +23951,15 @@
       </c>
       <c r="I422" s="70" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J422" s="70" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K422" s="70" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -24556,15 +24556,15 @@
       </c>
       <c r="I433" s="70" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J433" s="70" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K433" s="70" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -25271,15 +25271,15 @@
       </c>
       <c r="I446" s="70" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J446" s="70" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K446" s="70" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -25326,15 +25326,15 @@
       </c>
       <c r="I447" s="70" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J447" s="70" t="n">
-        <v>87.2</v>
+        <v>100</v>
       </c>
       <c r="K447" s="70" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -25381,15 +25381,15 @@
       </c>
       <c r="I448" s="70" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J448" s="70" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K448" s="70" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -25491,15 +25491,15 @@
       </c>
       <c r="I450" s="70" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J450" s="70" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K450" s="70" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -26096,15 +26096,15 @@
       </c>
       <c r="I461" s="70" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J461" s="70" t="n">
-        <v>80.7</v>
+        <v>100</v>
       </c>
       <c r="K461" s="70" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -26976,15 +26976,15 @@
       </c>
       <c r="I477" s="71" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J477" s="71" t="n">
-        <v>82.5</v>
+        <v>100</v>
       </c>
       <c r="K477" s="71" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -36221,15 +36221,15 @@
       </c>
       <c r="I666" s="68" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J666" s="68" t="n">
-        <v>28.9</v>
+        <v>35.6</v>
       </c>
       <c r="K666" s="68" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -36276,15 +36276,15 @@
       </c>
       <c r="I667" s="68" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J667" s="68" t="n">
-        <v>28.9</v>
+        <v>35.6</v>
       </c>
       <c r="K667" s="68" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -36331,15 +36331,15 @@
       </c>
       <c r="I668" s="68" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J668" s="68" t="n">
-        <v>35.6</v>
+        <v>41.1</v>
       </c>
       <c r="K668" s="68" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -36827,15 +36827,15 @@
       </c>
       <c r="I678" s="68" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J678" s="68" t="n">
-        <v>28.9</v>
+        <v>35.6</v>
       </c>
       <c r="K678" s="68" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -37078,15 +37078,15 @@
       </c>
       <c r="I683" s="68" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J683" s="68" t="n">
-        <v>28.9</v>
+        <v>35.6</v>
       </c>
       <c r="K683" s="68" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -37133,15 +37133,15 @@
       </c>
       <c r="I684" s="68" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J684" s="68" t="n">
-        <v>35.6</v>
+        <v>41.1</v>
       </c>
       <c r="K684" s="68" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -37188,15 +37188,15 @@
       </c>
       <c r="I685" s="68" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J685" s="68" t="n">
-        <v>35.6</v>
+        <v>41.1</v>
       </c>
       <c r="K685" s="68" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -37243,15 +37243,15 @@
       </c>
       <c r="I686" s="68" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J686" s="68" t="n">
-        <v>28.9</v>
+        <v>35.6</v>
       </c>
       <c r="K686" s="68" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -37298,15 +37298,15 @@
       </c>
       <c r="I687" s="68" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J687" s="68" t="n">
-        <v>35.6</v>
+        <v>41.1</v>
       </c>
       <c r="K687" s="68" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -37451,15 +37451,15 @@
       </c>
       <c r="I690" s="68" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J690" s="68" t="n">
-        <v>35.6</v>
+        <v>41.1</v>
       </c>
       <c r="K690" s="68" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -38883,15 +38883,15 @@
       <c r="H720" s="70" t="n"/>
       <c r="I720" s="70" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J720" s="70" t="n">
-        <v>20.2</v>
+        <v>28.9</v>
       </c>
       <c r="K720" s="70" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -38934,15 +38934,15 @@
       <c r="H721" s="70" t="n"/>
       <c r="I721" s="70" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J721" s="70" t="n">
-        <v>20.2</v>
+        <v>28.9</v>
       </c>
       <c r="K721" s="70" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -39036,15 +39036,15 @@
       <c r="H723" s="70" t="n"/>
       <c r="I723" s="70" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J723" s="70" t="n">
-        <v>20.2</v>
+        <v>28.9</v>
       </c>
       <c r="K723" s="70" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -39138,15 +39138,15 @@
       <c r="H725" s="70" t="n"/>
       <c r="I725" s="70" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J725" s="70" t="n">
-        <v>56.2</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="K725" s="70" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -39281,15 +39281,15 @@
       <c r="H728" s="70" t="n"/>
       <c r="I728" s="70" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J728" s="70" t="n">
-        <v>20.2</v>
+        <v>28.9</v>
       </c>
       <c r="K728" s="70" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -39790,15 +39790,15 @@
       </c>
       <c r="I739" s="70" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J739" s="70" t="n">
-        <v>57.1</v>
+        <v>64.3</v>
       </c>
       <c r="K739" s="70" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -40066,15 +40066,15 @@
       </c>
       <c r="I745" s="70" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J745" s="70" t="n">
-        <v>59.1</v>
+        <v>76</v>
       </c>
       <c r="K745" s="70" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -40697,15 +40697,15 @@
       </c>
       <c r="I758" s="70" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J758" s="70" t="n">
-        <v>64.90000000000001</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="K758" s="70" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -40957,15 +40957,15 @@
       <c r="H764" s="70" t="n"/>
       <c r="I764" s="70" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J764" s="70" t="n">
-        <v>57.1</v>
+        <v>64.3</v>
       </c>
       <c r="K764" s="70" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -41059,15 +41059,15 @@
       <c r="H766" s="70" t="n"/>
       <c r="I766" s="70" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J766" s="70" t="n">
-        <v>39</v>
+        <v>66.5</v>
       </c>
       <c r="K766" s="70" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -41151,15 +41151,15 @@
       <c r="H768" s="70" t="n"/>
       <c r="I768" s="70" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J768" s="70" t="n">
-        <v>20.2</v>
+        <v>28.9</v>
       </c>
       <c r="K768" s="70" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -41202,15 +41202,15 @@
       <c r="H769" s="70" t="n"/>
       <c r="I769" s="70" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J769" s="70" t="n">
-        <v>41.1</v>
+        <v>52.7</v>
       </c>
       <c r="K769" s="70" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>
@@ -41367,15 +41367,15 @@
       </c>
       <c r="I772" s="70" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="J772" s="70" t="n">
-        <v>56.7</v>
+        <v>85.7</v>
       </c>
       <c r="K772" s="70" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-28</t>
         </is>
       </c>
     </row>

</xml_diff>